<commit_message>
Sincronizacion 2026-09-25 (4): Ingresos sin el redondeo heredado
- Laminas de Ingresos regeneradas (regional, sexo y edad, provincial) sin el
  redondeo a 2 decimales que reproducia el CSV antiguo. Valores publicados
  identicos; deltas +-0,01; un empate desempatado (Arica / Promedio Regional).
- Payloads de Ingresos: Tarapaca 2024 pasa de 4,6% a 4,5%, como la capa.
- 1.216 XLSX de sexo y edad de otras dimensiones: identicos salvo la fecha.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_sexo_edad/plot_intra_i_ingr_a_2018_antofagasta.xlsx
+++ b/output/graficos_regionales_sexo_edad/plot_intra_i_ingr_a_2018_antofagasta.xlsx
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-18 09:02</t>
+    <t xml:space="preserve">2026-09-25 21:25</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -477,7 +477,7 @@
         <v>1164815.62</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>370698.87</v>
+        <v>370698.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>